<commit_message>
website content update - changes to estuaries, key messages, marine, species and terrestrial
</commit_message>
<xml_diff>
--- a/content/terrestrial/data/RLE index scores bootstrap.xlsx
+++ b/content/terrestrial/data/RLE index scores bootstrap.xlsx
@@ -415,7 +415,7 @@
         <v>0.8909090909090909</v>
       </c>
       <c r="F2">
-        <v>0.8089772727272727</v>
+        <v>0.8090909090909091</v>
       </c>
       <c r="G2">
         <v>0.9636363636363636</v>
@@ -445,7 +445,7 @@
         <v>0.8545454545454545</v>
       </c>
       <c r="F3">
-        <v>0.7636363636363637</v>
+        <v>0.759090909090909</v>
       </c>
       <c r="G3">
         <v>0.9363636363636364</v>
@@ -475,7 +475,7 @@
         <v>0.8545454545454545</v>
       </c>
       <c r="F4">
-        <v>0.7681818181818182</v>
+        <v>0.7636363636363637</v>
       </c>
       <c r="G4">
         <v>0.9363636363636364</v>
@@ -625,10 +625,10 @@
         <v>0.8111111111111111</v>
       </c>
       <c r="F9">
-        <v>0.6555555555555556</v>
+        <v>0.6666666666666667</v>
       </c>
       <c r="G9">
-        <v>0.9555555555555556</v>
+        <v>0.9333333333333333</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -895,10 +895,10 @@
         <v>0.6333333333333333</v>
       </c>
       <c r="F18">
-        <v>0.5714285714285714</v>
+        <v>0.5698412698412698</v>
       </c>
       <c r="G18">
-        <v>0.6968253968253968</v>
+        <v>0.6984126984126984</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         <v>0.553968253968254</v>
       </c>
       <c r="G19">
-        <v>0.680952380952381</v>
+        <v>0.6825396825396826</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -955,10 +955,10 @@
         <v>0.6174603174603175</v>
       </c>
       <c r="F20">
-        <v>0.5523809523809524</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="G20">
-        <v>0.680992063492063</v>
+        <v>0.6793650793650794</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -985,10 +985,10 @@
         <v>0.6174603174603175</v>
       </c>
       <c r="F21">
-        <v>0.5523809523809524</v>
+        <v>0.553968253968254</v>
       </c>
       <c r="G21">
-        <v>0.6825396825396826</v>
+        <v>0.680952380952381</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1015,10 +1015,10 @@
         <v>0.8465753424657534</v>
       </c>
       <c r="F22">
-        <v>0.7890410958904109</v>
+        <v>0.7863013698630137</v>
       </c>
       <c r="G22">
-        <v>0.904109589041096</v>
+        <v>0.9014383561643825</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1045,10 +1045,10 @@
         <v>0.8191780821917808</v>
       </c>
       <c r="F23">
-        <v>0.7534246575342466</v>
+        <v>0.7561643835616438</v>
       </c>
       <c r="G23">
-        <v>0.8821917808219178</v>
+        <v>0.8794520547945206</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1105,10 +1105,10 @@
         <v>0.8082191780821918</v>
       </c>
       <c r="F25">
-        <v>0.7397260273972603</v>
+        <v>0.7424657534246575</v>
       </c>
       <c r="G25">
-        <v>0.8684931506849315</v>
+        <v>0.8712328767123287</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -1378,7 +1378,7 @@
         <v>0.8617021276595744</v>
       </c>
       <c r="G34">
-        <v>0.951063829787234</v>
+        <v>0.948936170212766</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
         <v>0.8872340425531915</v>
       </c>
       <c r="F35">
-        <v>0.8361702127659575</v>
+        <v>0.8340425531914893</v>
       </c>
       <c r="G35">
         <v>0.9340425531914893</v>
@@ -1435,10 +1435,10 @@
         <v>0.874468085106383</v>
       </c>
       <c r="F36">
-        <v>0.823404255319149</v>
+        <v>0.8212765957446808</v>
       </c>
       <c r="G36">
-        <v>0.9234042553191489</v>
+        <v>0.9212765957446809</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -1468,7 +1468,7 @@
         <v>0.8212765957446808</v>
       </c>
       <c r="G37">
-        <v>0.9234042553191489</v>
+        <v>0.925531914893617</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -1495,7 +1495,7 @@
         <v>0.93125</v>
       </c>
       <c r="F38">
-        <v>0.875</v>
+        <v>0.871875</v>
       </c>
       <c r="G38">
         <v>0.978125</v>
@@ -1558,7 +1558,7 @@
         <v>0.85625</v>
       </c>
       <c r="G40">
-        <v>0.96875</v>
+        <v>0.971875</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -1585,10 +1585,10 @@
         <v>0.91875</v>
       </c>
       <c r="F41">
-        <v>0.85625</v>
+        <v>0.859375</v>
       </c>
       <c r="G41">
-        <v>0.96875</v>
+        <v>0.971953124999999</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -1610,10 +1610,10 @@
         <v>0.8215982721382289</v>
       </c>
       <c r="F42">
-        <v>0.7930777537796976</v>
+        <v>0.7952483801295896</v>
       </c>
       <c r="G42">
-        <v>0.8479481641468682</v>
+        <v>0.847095032397408</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -1635,10 +1635,10 @@
         <v>0.7987041036717063</v>
       </c>
       <c r="F43">
-        <v>0.7706263498920086</v>
+        <v>0.7693304535637149</v>
       </c>
       <c r="G43">
-        <v>0.827656587473002</v>
+        <v>0.8263606911447082</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -1660,10 +1660,10 @@
         <v>0.7961123110151188</v>
       </c>
       <c r="F44">
-        <v>0.767170626349892</v>
+        <v>0.7675917926565874</v>
       </c>
       <c r="G44">
-        <v>0.824622030237581</v>
+        <v>0.8241900647948164</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -1685,7 +1685,7 @@
         <v>0.7943844492440605</v>
       </c>
       <c r="F45">
-        <v>0.7658747300215982</v>
+        <v>0.7650107991360691</v>
       </c>
       <c r="G45">
         <v>0.8233261339092872</v>

</xml_diff>